<commit_message>
Add driver pay mode: per-mile ($/mile) or per-hour; per-mile is default to avoid time-padding
</commit_message>
<xml_diff>
--- a/results/sample_ortools_report.xlsx
+++ b/results/sample_ortools_report.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -638,30 +638,52 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Driver wage per hour ($)</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>20</v>
+          <t>Labor mode</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>per hour ($/h)</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Management fee per vehicle ($)</t>
+          <t>Driver wage per distance ($/mile)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>15</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Driver wage per hour ($/h)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Management fee per vehicle ($)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Deductible per vehicle ($)</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B25" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>